<commit_message>
Schema onerisi QAPage yerine FAQPage: Google yonergesi ve FAQ rich result durumu
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
+++ b/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Tek bir soru ve onun cevabını taşıyan sayfaları tanımlayan schema tipi.</t>
+          <t>Kullanıcıların bir soruya cevap ekleyebildiği sayfaları (forum gibi) tanımlayan schema tipi; site tarafından yazılan tek cevaplı sayfalarda kullanılmaz.</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Bir sayfadaki birden fazla soru-cevap bloğunu tanımlayan schema tipi.</t>
+          <t>Sitenin kendi yazdığı soru-cevap içeriğini tanımlayan schema tipi; tek soru ya da birden fazla soru taşıyabilir.</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Soru-cevap yapısının QAPage schema ile işaretlenmesi</t>
+          <t>Soru-cevap yapısının FAQPage schema ile işaretlenmesi</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -1905,20 +1905,19 @@
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>Destek soru şablonuna QAPage tipinde JSON-LD eklenmelidir; soru metni H1'den, cevap metni cevap gövdesinden sunucu tarafında üretilmelidir. Mevcut BreadcrumbList ve WebPage blokları korunmalıdır. Ticari sayfaların SSS bölümlerinde (ör. /esim, /turkcellailem/) FAQPage kullanılmalıdır. İşaretleme, soft 404 düzeltmesi tamamlanmadan yaygınlaştırılmamalıdır; aksi halde başka sayfanın içeriğini gösteren adresler de soru-cevap olarak işaretlenir.</t>
+          <t>Destek soru şablonuna FAQPage tipinde JSON-LD eklenmelidir; tek Question içerir, soru metni H1'den, cevap metni cevap gövdesinden sunucu tarafında üretilmelidir. QAPage kullanılmamalıdır: Google yönergesine göre QAPage yalnızca kullanıcıların cevap ekleyebildiği sayfalar içindir; sitenin yazdığı tek cevaplı sayfalar bu kapsamda değildir. FAQ rich result Mayıs 2026'dan bu yana Google Arama'da gösterilmediği için işaretlemeden rich result beklenmez; amaç soru ve cevabın arama motorlarına ve yapay zeka araçlarına kodla bildirilmesidir. Mevcut BreadcrumbList ve WebPage blokları korunmalıdır. Ticari sayfaların SSS bölümlerinde (ör. /esim, /turkcellailem/) her soru ayrı Question olarak FAQPage'e eklenmelidir. İşaretleme, soft 404 düzeltmesi tamamlanmadan yaygınlaştırılmamalıdır; aksi halde başka sayfanın içeriğini gösteren adresler de soru-cevap olarak işaretlenir.</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
           <t>{
   "@context": "https://schema.org",
-  "@type": "QAPage",
-  "mainEntity": {
+  "@type": "FAQPage",
+  "mainEntity": [{
     "@type": "Question",
     "name": "&lt;H1&gt;",
-    "answerCount": 1,
-    "acceptedAnswer": {"@type": "Answer", "text": "&lt;cevap gövdesi&gt;", "url": "&lt;sayfa adresi&gt;"}
-  }
+    "acceptedAnswer": {"@type": "Answer", "text": "&lt;cevap gövdesinin düz metni&gt;"}
+  }]
 }</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Soft 404 hedefleri Search Console sorgularina ve icerige gore yeniden belirlendi; Soft 404 - tekrar eden sayfalar ve Duplicate adresler adlandirmasi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
+++ b/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mevcut Sayfa Güçlendirme" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sitemap Dışı Adresler" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doğrulanacak Bilgiler" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mükerrer Sayfalar" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duplicate Adresler" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rakip Karşılaştırması" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Eşleştirme" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terim Sözlüğü" sheetId="10" state="visible" r:id="rId10"/>
@@ -24,10 +24,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mevcut Sayfa Güçlendirme'!$A$4:$O$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sitemap Dışı Adresler'!$A$4:$L$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Doğrulanacak Bilgiler'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Mükerrer Sayfalar'!$A$4:$G$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Duplicate Adresler'!$A$4:$G$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Rakip Karşılaştırması'!$A$4:$K$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Prompt Eşleştirme'!$A$4:$G$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Terim Sözlüğü'!$A$4:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Terim Sözlüğü'!$A$4:$C$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -822,7 +822,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Soft 404 adresi</t>
+          <t xml:space="preserve">  Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="B17" s="6">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B21" s="6">
-        <f>COUNTA('Mükerrer Sayfalar'!C5:C1000)</f>
+        <f>COUNTA('Duplicate Adresler'!C5:C1000)</f>
         <v/>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1005,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1204,12 +1204,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Duplicate adres</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Aynı içeriğe birden çok adresten ulaşılabildiğinde 'asıl adres budur' diyen işaret.</t>
+          <t>Aynı başlığı ve cevabı taşıyan birden fazla adres; tek adreste birleştirilmesi önerilir.</t>
         </is>
       </c>
     </row>
@@ -1221,12 +1221,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Bir adresin kalıcı olarak başka bir adrese taşındığını bildiren yönlendirme.</t>
+          <t>Aynı içeriğe birden çok adresten ulaşılabildiğinde 'asıl adres budur' diyen işaret.</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>404 / 410</t>
+          <t>301</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Sayfanın bulunamadığını (404) ya da kalıcı olarak kaldırıldığını (410) bildiren yanıt kodu.</t>
+          <t>Bir adresin kalıcı olarak başka bir adrese taşındığını bildiren yönlendirme.</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>404 / 410</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Gerçekte var olmayan bir adresin hata kodu yerine 200 dönüp başka bir içerik göstermesi.</t>
+          <t>Sayfanın bulunamadığını (404) ya da kalıcı olarak kaldırıldığını (410) bildiren yanıt kodu.</t>
         </is>
       </c>
     </row>
@@ -1272,12 +1272,12 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Sitemap</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Sitenin arama motorlarına bildirdiği sayfa listesi dosyası.</t>
+          <t>Gerçekte var olmayan bir adresin hata kodu yerine 200 dönüp başka bir sayfanın içeriğini tekrar etmesi.</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Internal linking</t>
+          <t>Sitemap</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Site içindeki sayfaların birbirine verdiği bağlantılar.</t>
+          <t>Sitenin arama motorlarına bildirdiği sayfa listesi dosyası.</t>
         </is>
       </c>
     </row>
@@ -1306,29 +1306,29 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>SERP</t>
+          <t>Internal linking</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Arama sonuç sayfası.</t>
+          <t>Site içindeki sayfaların birbirine verdiği bağlantılar.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>Yapısal veri</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Schema / JSON-LD</t>
+          <t>SERP</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Sayfadaki içeriğin ne olduğunu arama motoruna makine tarafından okunabilir biçimde bildiren etiket.</t>
+          <t>Arama sonuç sayfası.</t>
         </is>
       </c>
     </row>
@@ -1340,12 +1340,12 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>QAPage</t>
+          <t>Schema / JSON-LD</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Kullanıcıların bir soruya cevap ekleyebildiği sayfaları (forum gibi) tanımlayan schema tipi; site tarafından yazılan tek cevaplı sayfalarda kullanılmaz.</t>
+          <t>Sayfadaki içeriğin ne olduğunu arama motoruna makine tarafından okunabilir biçimde bildiren etiket.</t>
         </is>
       </c>
     </row>
@@ -1357,29 +1357,29 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>FAQPage</t>
+          <t>QAPage</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Sitenin kendi yazdığı soru-cevap içeriğini tanımlayan schema tipi; tek soru ya da birden fazla soru taşıyabilir.</t>
+          <t>Kullanıcıların bir soruya cevap ekleyebildiği sayfaları (forum gibi) tanımlayan schema tipi; site tarafından yazılan tek cevaplı sayfalarda kullanılmaz.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>GEO</t>
+          <t>Yapısal veri</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>GEO</t>
+          <t>FAQPage</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>İçeriğin yapay zeka cevaplarında kaynak olarak seçilmesine yönelik çalışma.</t>
+          <t>Sitenin kendi yazdığı soru-cevap içeriğini tanımlayan schema tipi; tek soru ya da birden fazla soru taşıyabilir.</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>AI Overview</t>
+          <t>GEO</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Google'ın arama sonuçlarının üstünde gösterdiği yapay zeka özet paneli.</t>
+          <t>İçeriğin yapay zeka cevaplarında kaynak olarak seçilmesine yönelik çalışma.</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>AI Overview</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>People Also Ask; arama sonuçlarındaki İlgili sorular paneli.</t>
+          <t>Google'ın arama sonuçlarının üstünde gösterdiği yapay zeka özet paneli.</t>
         </is>
       </c>
     </row>
@@ -1425,29 +1425,29 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Prompt</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Kullanıcının yapay zeka aracına yazdığı soru ya da talep.</t>
+          <t>People Also Ask; arama sonuçlarındaki İlgili sorular paneli.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>Teknik</t>
+          <t>GEO</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>USSD kodu</t>
+          <t>Prompt</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Telefonun tuş takımından girilen ve * ile # içeren servis kodu (ör. *#06#).</t>
+          <t>Kullanıcının yapay zeka aracına yazdığı soru ya da talep.</t>
         </is>
       </c>
     </row>
@@ -1459,17 +1459,34 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
+          <t>USSD kodu</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Telefonun tuş takımından girilen ve * ile # içeren servis kodu (ör. *#06#).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Teknik</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
           <t>APN</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Telefonun mobil internete bağlanmak için kullandığı erişim noktası ayarı.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C28"/>
+  <autoFilter ref="A4:C29"/>
   <mergeCells count="1">
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1632,12 +1649,12 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Var olmayan destek adreslerinin 200 dönüp başka sayfanın içeriğini göstermesi (soft 404)</t>
+          <t>Soft 404 - tekrar eden sayfalar: yayında olmayan adreslerin başka sayfanın içeriğini göstermesi</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Geçerli bir kategori ve alt bölüm altında yayında olmayan bir soru adresi istendiğinde sunucu 200 status code döndürmekte, alt bölümdeki başka bir sayfanın içeriğini göstermekte, adresin kendisine canonical vermekte ve index,follow taşımaktadır (test: /destek/tarife-ve-paketler/konusma/bu-sayfa-yok-deneme-xyz, 14 Eyl 2026). Geçersiz kategori ya da alt bölüm altında adres doğru biçimde 404 dönmektedir. Search Console'da 1 Eyl 2025 - 31 Ağu 2026 penceresinde bu davranışı gösteren 30 adres görülmüştür: 26 adres başka bir sayfanın içeriğini göstermekte (215.336 impression, 6.790 tıklama), 4 adres ise gerçek bir sayfanın yazım varyantı olarak kopyasını sunmaktadır (95.306 impression). Toplam 310.642 impression.</t>
+          <t>Geçerli bir kategori ve alt bölüm altında yayında olmayan bir soru adresi istendiğinde sunucu 200 status code döndürmekte, alt bölümdeki başka bir sayfanın içeriğini göstermekte, adresin kendisine canonical vermekte ve index,follow taşımaktadır (test: /destek/tarife-ve-paketler/konusma/bu-sayfa-yok-deneme-xyz, 14 Eyl 2026). Geçersiz kategori ya da alt bölüm altında adres doğru biçimde 404 dönmektedir. Search Console'da 1 Eyl 2025 - 31 Ağu 2026 penceresinde bu davranışı gösteren 28 adres görülmüştür: 24 adres başka bir sayfanın içeriğini tekrar etmekte (212.184 impression, 5.168 tıklama), 4 adres ise gerçek bir sayfanın yazım varyantı olarak kopyasını sunmaktadır (95.306 impression). Toplam 307.490 impression. Şikayet talebi oluşturma ve Pasaj satıcı sayfaları kendi içeriğini gösterdiği için bu listeye alınmamıştır.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
@@ -1647,7 +1664,7 @@
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>Var olmayan destek adresleri 404 (kalıcı olarak kaldırılanlar için 410) status code döndürmelidir. Kaldırılmış soru sayfalarının adresleri, sorunun güncel cevabını veren sayfaya 301 ile yönlendirilmelidir (adres bazlı liste 'Kaldırılmış soru sayfaları' maddesinde). Yazım varyantı adresler gerçek adrese 301 ile yönlendirilmeli; canonical, istenen adrese değil gösterilen içeriğin asıl adresine verilmelidir. Yeni önerilen sayfalar yayına alınmadan önce önerilen adreslerin bu davranış nedeniyle zaten 200 döndüğü dikkate alınmalıdır.</t>
+          <t>Var olmayan destek adresleri 404 (kalıcı olarak kaldırılanlar için 410) status code döndürmelidir. Kaldırılmış soru sayfalarının adresleri, sorunun güncel cevabını veren sayfaya 301 ile yönlendirilmelidir (adres bazlı liste 'Kaldırılmış soru sayfaları' maddesinde ve aksiyon listesinin Soft 404 - tekrar eden sayfalar sekmesinde). Yazım varyantı adresler gerçek adrese 301 ile yönlendirilmeli; canonical, istenen adrese değil gösterilen içeriğin asıl adresine verilmelidir. Yeni önerilen sayfalar yayına alınmadan önce önerilen adreslerin bu davranış nedeniyle zaten 200 döndüğü dikkate alınmalıdır.</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -1664,7 +1681,7 @@
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>30 adres · 310.642 impression (Search Console, 1 Eyl 2025 - 31 Ağu 2026)</t>
+          <t>28 adres · 307.490 impression (Search Console, 1 Eyl 2025 - 31 Ağu 2026) + şablon kuralı</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1716,7 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Adreslerin sitemap dosyasına eklenmesi, H1 bulunmayan araç sayfalarına sayfa konusunu tarif eden bir H1 eklenmesi ve 'Numaramı nasıl taşıyabilirim?' sayfasının dijital başvuru kanallarını da içerecek şekilde güncellenmesi önerilir. '/destek/turkcell-akademi' adresi destek ana sayfasına yönlendiği için sitemap'e eklenmemelidir.</t>
+          <t>Adreslerin sitemap dosyasına eklenmesi ve H1 bulunmayan araç ve form sayfalarına (şikayet talebi oluşturma dahil) sayfa konusunu tarif eden title ve H1 eklenmesi önerilir. 'Numaramı nasıl taşıyabilirim?' sayfası noindex ve canonical'i paket seçimi sayfasına veriyor; canonical'in yönlenen /trc/turkcellli-olmak/paket-secimi yerine son adrese (/turkcellli-olmak/paket-secimi) verilmesi, sayfanın sitemap'e eklenmemesi önerilir. '/destek/turkcell-akademi' adresi destek ana sayfasına yönlendiği için sitemap'e eklenmemelidir.</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1751,26 +1768,39 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>Aşağıdaki eşleme uygulanmalıdır. Yeniden açılacak iki adres (paket aşım ücreti ve tarife bilgisi sorgulama), arama geçmişini korumak için aynı adreste yeni içerikle yayınlanmalıdır. Yönlendirilecek adreslerde 301 hedefi, gösterilen içeriğin değil sorunun cevabını veren sayfanın adresi olmalıdır.</t>
+          <t>Aşağıdaki eşleme uygulanmalıdır. Hedefler, her adresin Search Console sorguları ve hedef sayfanın canlı içeriği karşılaştırılarak belirlenmiştir; 301 hedefi, adreste bugün görünen içeriğin değil, adresin aldığı sorguları cevaplayan sayfanın adresidir. Paket aşım ücreti adresi, arama geçmişini korumak için aynı adreste yeni içerikle yayınlanmalıdır.</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>/destek/online-alisveris/odeme/paycell-dijital-para-ile-odeme-secenegi-nedir · 73.878 impression → 301 → /servisler/uygulamalar/paycell ('paycell nedir' talebi)
+          <t>/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odenmedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir · 95.156 impression → 301 → /destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odemedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir
+/destek/online-alisveris/odeme/paycell-dijital-para-ile-odeme-secenegi-nedir · 73.878 impression → 301 → /servisler/uygulamalar/paycell
 /destek/hizmet-kanallarimiz/musteri-hizmetleri/bip-turkcell-musteri-hizmetleri · 34.940 impression → 301 → /destek/hizmet-kanallarimiz/musteri-hizmetleri/532-turkcell-musteri-hizmetleri
-/destek/kampanya/kampanyalar-faturali/numara-tasima-nedir · 31.695 impression → 301 → /destek/turkcellli-olmak/numara-tasima/numara-tasima-nedir
-/destek/tarife-ve-paketler/konusma/paket-asim-ucreti-nedir · 24.167 impression → İçerik olarak yeniden açılmalı: yeni sayfa seti 'Paket aşımı nedir, paket bittikten sonra aşım nasıl kapatılır?'
+/destek/kampanya/kampanyalar-faturali/numara-tasima-nedir · 31.695 impression → 301 → /turkcellli-olmak/paket-secimi
+/destek/tarife-ve-paketler/konusma/paket-asim-ucreti-nedir · 24.167 impression → aynı adreste yeni içerikle yeniden açılış
 /destek/online-alisveris/odeme/faturama-yansit-odeme-secenegi-nedir · 11.454 impression → 301 → /servisler/arama-fatura-tl/turkcellmobilodeme
-/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim · 6.518 impression → İçerik olarak yeniden açılmalı: yeni sayfa seti 'Tarife bilgilerimi nasıl sorgularım, mevcut tarifem nasıl öğrenilir?'
-/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-servislerim-sayfasindan-hangi-bilgilere-ulasabilirim · 5.510 impression → 301 → /destek/islem-merkezi/hat-ozetim/hat-ozetim-nedir
-/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-kampanyalarimla-hangi-islemleri-yapabilirim · 5.152 impression → 301 → /destek/islem-merkezi/hat-ozetim/hat-ozetim-nedir
-/destek/servisler-ve-internet/servisler/avans-tl-nedir-nasil-abone-olurum · 4.580 impression → Servisin yayında olup olmadığı marka tarafından teyit edilmeli; yayında değilse 410
-/destek/kampanya/kampanyalar-faturali/numarami-nasil-tasiyabilirim · 4.541 impression → 301 → /destek/turkcellli-olmak/numara-tasima/numarami-nasil-tasiyabilirim
-/destek/tuketici-sikayetleri/sikayet-talebi-olusturma · 3.123 impression → H1 ve title boş dönüyor; form sayfasının güncel adresi teyit edilmeli (1.614 tıklama alıyor)
+/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim · 6.518 impression → 301 → /paket-ve-tarifeler
+/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-servislerim-sayfasindan-hangi-bilgilere-ulasabilirim · 5.510 impression → 301 → /destek/islem-merkezi
+/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-kampanyalarimla-hangi-islemleri-yapabilirim · 5.152 impression → 301 → /destek/islem-merkezi
+/destek/servisler-ve-internet/servisler/avans-tl-nedir-nasil-abone-olurum · 4.580 impression → 410 dönmesi (Avans TL servis sayfası da kaldırılmış)
+/destek/kampanya/kampanyalar-faturali/numarami-nasil-tasiyabilirim · 4.541 impression → 301 → /turkcellli-olmak/paket-secimi
 /destek/turkcellli-olmak/turkcellli-olmak/nasil-hazirkart-alirim · 2.934 impression → 301 → /destek/turkcellli-olmak/numara-tasima/nasil-hazirkart-alirim
+/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimlerine-nereden-ulasabilirim · 2.481 impression → 301 → https://tag.turkcell.com.tr/
 /destek/servisler-ve-internet/servisler/kredi-transfer-nedir · 1.268 impression → 301 → /destek/hattiniz/hazirkart/kreditransfer-nedir
-/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim · 1.227 impression → 301 → /servisler/arama-fatura-tl/turkcellmobilodeme
-/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi · 779 impression → 301 → /destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
+/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim · 1.227 impression → 301 → /servisler/arama-fatura-tl/yonlendir
+/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi · 779 impression → 301 → /destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi
+/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim · 382 impression → 301 → /destek/islem-merkezi
+/destek/sosyal-destek-iletisim · 257 impression → 301 → /sosyal-destek
+/destek/turkcell-akademi/sikca-sorulan-sorular/mevcut-egitimlerden-baska-egitimler-olacak-mi · 172 impression → 301 → https://tag.turkcell.com.tr/
+/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim · 145 impression → 404 ya da 410 dönmesi (karşılayan sayfa yok)
+/destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir · 129 impression → 301 → /destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir
+/destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim · 55 impression → 301 → /destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim
+/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak- · 33 impression → 301 → /kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-gelen-ve-gelen-giden-iletisime-ne-kadar-sureyle-kapatabilirim-ve-faturama-herhangi-bir-ucret-yansir-m
+/destek/islem-merkezi/ayarlarim/hat-iptalimi-nasil-gerceklestirebilirim · 14 impression → 301 → /destek/hattiniz/abonelik-islemleri/hattimi-nasil-iptal-ettirebilirim
+/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken · 14 impression → 301 → /destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir
+/destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir · 7 impression → 301 → /destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir
+/destek/hizmet-kanallarimiz/musteri-hizmetleri/gencaver · 1 impression → 404 ya da 410 dönmesi
+/destek/online-alisveris · 1 impression → 301 → /destek/online-alisveris</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
@@ -1865,7 +1895,7 @@
           <t>Kurumsal: /kurumsal/destek/hattiniz/hazirkart/telsiz-kullanim-ucreti-nedir
 Bireysel: /destek/hattiniz/hazirkart/telsiz-kullanim-ucreti
 Kurumsal: /kurumsal/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim
-Bireysel: önerilen /destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim (yeniden açılış)</t>
+Bireysel: önerilen /destek/tarife-ve-paketler/konusma/mevcut-tarifemi-nasil-ogrenebilirim (yeniden açılış)</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
@@ -1943,7 +1973,7 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Aynı içeriği taşıyan adreslerin birleştirilmesi</t>
+          <t>Duplicate adreslerin birleştirilmesi (aynı içeriği taşıyan adresler)</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -4244,7 +4274,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/mevcut-tarifemi-nasil-ogrenebilirim</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
@@ -4300,7 +4330,7 @@
 • Search Console: 25.689 impression · 1.390 click · ağırlıklı konum 4,6
 • Tıklama alan sayfa: https://www.turkcell.com.tr/kurumsal/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim
 • Bireysel destekte bu soruyu cevaplayan sayfa bir dönem yayındaydı; adres bugün başka bir sayfanın içeriğini gösterdiği için talep kurumsal kopyaya kaymaktadır.
-• Adres bugün başka bir sayfanın içeriğini göstermekte ancak arama talebi almaya devam etmektedir; sayfanın aynı adreste yeniden açılması önerilir.</t>
+• Eski bireysel adresin kendi sorguları genel paket ve tarife araması olduğundan eski adres /paket-ve-tarifeler sayfasına yönlendirilir; sayfa yeni adreste açılır.</t>
         </is>
       </c>
       <c r="Q21" s="14" t="inlineStr">
@@ -7958,7 +7988,7 @@
               <color rgb="00FF7B52"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Mükerrer adresler: </t>
+            <t xml:space="preserve">Duplicate adresler: </t>
           </r>
           <r>
             <rPr>
@@ -8025,7 +8055,7 @@
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>Mükerrer adresler</t>
+          <t>Duplicate adresler</t>
         </is>
       </c>
       <c r="H4" s="10" t="inlineStr">
@@ -12315,7 +12345,7 @@
               <color rgb="0010332F"/>
               <sz val="10"/>
             </rPr>
-            <t>Sayfa yayında ve doğru içeriği gösteriyor; Önerilen işlem sütunundaki düzenleme uygulanır.</t>
+            <t>Sayfa yayında ve kendi içeriğini gösteriyor; Önerilen işlem sütunundaki düzenleme uygulanır.</t>
           </r>
           <r>
             <t>
@@ -12328,7 +12358,7 @@
               <color rgb="00FF7B52"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Soft 404: </t>
+            <t xml:space="preserve">Soft 404 - tekrar eden sayfa: </t>
           </r>
           <r>
             <rPr>
@@ -12336,7 +12366,7 @@
               <color rgb="0010332F"/>
               <sz val="10"/>
             </rPr>
-            <t>Adres yayında değil ama 404 yerine 200 dönüyor. Görünen H1 ve cevap başka bir sayfaya aittir (asıl adresi İçeriğin asıl adresi sütununda); canonical açılan adresin kendisine veriliyor ve adres indekslenebilir durumda.</t>
+            <t>Adres yayında değil ama 404 yerine 200 dönüyor ve başka bir sayfanın içeriğini tekrar ediyor. Görünen H1 ve cevap başka bir sayfaya aittir (asıl adresi İçeriğin asıl adresi sütununda); canonical açılan adresin kendisine veriliyor ve adres indekslenebilir durumda.</t>
           </r>
           <r>
             <t>
@@ -12582,7 +12612,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>noindex etiketinin kaldırılması, canonical'in kendi adresine verilmesi ve sitemap'e eklenmesi</t>
+          <t>Canonical'in yönlenen /trc/turkcellli-olmak/paket-secimi yerine son adrese (/turkcellli-olmak/paket-secimi) verilmesi; sayfa noindex olduğu için sitemap'e eklenmemesi</t>
         </is>
       </c>
     </row>
@@ -12759,7 +12789,7 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/kurumsal/destek/cihaz-satisi</t>
+          <t>https://www.turkcell.com.tr/destek/tuketici-sikayetleri/sikayet-talebi-olusturma</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
@@ -12777,12 +12807,12 @@
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>Cihaz Satışı</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>Cihaz Satışı</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -12791,14 +12821,14 @@
         </is>
       </c>
       <c r="J11" s="19" t="n">
-        <v>35</v>
+        <v>3123</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>11</v>
+        <v>1614</v>
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>Sitemap'e eklenmesi</t>
+          <t>Çalışan şikayet formu; title ve H1 boş dönüyor. Title ve H1 eklenmesi, sitemap'e eklenmesi</t>
         </is>
       </c>
     </row>
@@ -12806,14 +12836,14 @@
       <c r="A12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404 · yazım varyantı</t>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Açık sayfa · sitemap'te yok</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odenmedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
+          <t>https://www.turkcell.com.tr/kurumsal/destek/cihaz-satisi</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
@@ -12831,28 +12861,28 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>Faturamı Son Ödeme Tarihinde Ödenmediğimde Hattımın Kısıtlanma ve Durdurma Süre ve Süreçleri Nelerdir?</t>
+          <t>Cihaz Satışı</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>Faturamı son ödeme tarihinde ödemediğimde hattımın kısıtlanma ve durdurma süre ve süreçleri nelerdir?</t>
+          <t>Cihaz Satışı</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odemedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J12" s="19" t="n">
-        <v>95156</v>
+        <v>35</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>8406</v>
+        <v>11</v>
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odemedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
+          <t>Sitemap'e eklenmesi</t>
         </is>
       </c>
     </row>
@@ -12860,14 +12890,14 @@
       <c r="A13" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404</t>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Açık sayfa · sitemap'te yok</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/paycell-dijital-para-ile-odeme-secenegi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/online-alisveris/turkcell-pasaj/turkcell-pasajda-satici-olmak-istiyorum-nereye-basvurabilirim</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
@@ -12880,33 +12910,33 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>noindex,nofollow</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>Paycell Dijital Para ile Ödeme Seçeneği Nedir?</t>
+          <t>Turkcell Pasaj’da Satıcı Olmak İstiyorum, Nereye Başvurabilirim?</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>Ödeme seçeneklerim nelerdir?</t>
+          <t>Turkcell Pasaj'da satıcı olmak istiyorum.</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/odeme-seceneklerim-nelerdir</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J13" s="19" t="n">
-        <v>73878</v>
+        <v>29</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>2239</v>
+        <v>8</v>
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/servisler/uygulamalar/paycell</t>
+          <t>Kendi içeriğini gösteriyor, bilinçli olarak noindex; işlem gerekmiyor</t>
         </is>
       </c>
     </row>
@@ -12916,12 +12946,12 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/bip-turkcell-musteri-hizmetleri</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odenmedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
@@ -12939,28 +12969,28 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>BiP Turkcell Müşteri Hizmetleri | Turkcell Destek</t>
+          <t>Faturamı Son Ödeme Tarihinde Ödenmediğimde Hattımın Kısıtlanma ve Durdurma Süre ve Süreçleri Nelerdir?</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Hizmet</t>
+          <t>Faturamı son ödeme tarihinde ödemediğimde hattımın kısıtlanma ve durdurma süre ve süreçleri nelerdir?</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/turkcell-hizmet</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odemedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
         </is>
       </c>
       <c r="J14" s="19" t="n">
-        <v>34940</v>
+        <v>95156</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>277</v>
+        <v>8406</v>
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/532-turkcell-musteri-hizmetleri</t>
+          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/faturali/faturami-son-odeme-tarihinde-odemedigimde-hattimin-kisitlanma-ve-durdurma-sure-ve-surecleri-nelerdir</t>
         </is>
       </c>
     </row>
@@ -12970,12 +13000,12 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numara-tasima-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/paycell-dijital-para-ile-odeme-secenegi-nedir</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
@@ -12993,28 +13023,28 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>Numara Taşıma Kampanyaları Nelerdir?</t>
+          <t>Paycell Dijital Para ile Ödeme Seçeneği Nedir?</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>Numaramı taşımak ücretli midir?</t>
+          <t>Ödeme seçeneklerim nelerdir?</t>
         </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
+          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/odeme-seceneklerim-nelerdir</t>
         </is>
       </c>
       <c r="J15" s="19" t="n">
-        <v>31695</v>
+        <v>73878</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>729</v>
+        <v>2239</v>
       </c>
       <c r="L15" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numara-tasima-nedir</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/servisler/uygulamalar/paycell</t>
         </is>
       </c>
     </row>
@@ -13024,12 +13054,12 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/paket-asim-ucreti-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/bip-turkcell-musteri-hizmetleri</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
@@ -13047,28 +13077,28 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Paket Aşım Ücreti Nedir? | Turkcell Destek</t>
+          <t>BiP Turkcell Müşteri Hizmetleri | Turkcell Destek</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
+          <t>Turkcell Hizmet</t>
         </is>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/turkcell-hizmet</t>
         </is>
       </c>
       <c r="J16" s="19" t="n">
-        <v>24167</v>
+        <v>34940</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>202</v>
+        <v>277</v>
       </c>
       <c r="L16" s="14" t="inlineStr">
         <is>
-          <t>Aynı adreste yeni içerikle yeniden açılması</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/532-turkcell-musteri-hizmetleri</t>
         </is>
       </c>
     </row>
@@ -13078,12 +13108,12 @@
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/faturama-yansit-odeme-secenegi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numara-tasima-nedir</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
@@ -13101,28 +13131,28 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>Faturama Yansıt Ödeme Seçeneği Nedir?</t>
+          <t>Numara Taşıma Kampanyaları Nelerdir?</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>Ödeme seçeneklerim nelerdir?</t>
+          <t>Numaramı taşımak ücretli midir?</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/odeme-seceneklerim-nelerdir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
         </is>
       </c>
       <c r="J17" s="19" t="n">
-        <v>11454</v>
+        <v>31695</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>944</v>
+        <v>729</v>
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/servisler/arama-fatura-tl/turkcellmobilodeme</t>
+          <t>301 ile yönlendirilmesi (sorgular numara taşıma kampanyası ve tarifesi arıyor): https://www.turkcell.com.tr/turkcellli-olmak/paket-secimi</t>
         </is>
       </c>
     </row>
@@ -13132,12 +13162,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/paket-asim-ucreti-nedir</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
@@ -13155,24 +13185,24 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
+          <t>Paket Aşım Ücreti Nedir? | Turkcell Destek</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
           <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
-        </is>
-      </c>
       <c r="I18" s="14" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="J18" s="19" t="n">
-        <v>6518</v>
+        <v>24167</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>66</v>
+        <v>202</v>
       </c>
       <c r="L18" s="14" t="inlineStr">
         <is>
@@ -13186,12 +13216,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-servislerim-sayfasindan-hangi-bilgilere-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/faturama-yansit-odeme-secenegi-nedir</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
@@ -13209,28 +13239,28 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>Servislerim Sayfasında Hangi Bilgiler Var?</t>
+          <t>Faturama Yansıt Ödeme Seçeneği Nedir?</t>
         </is>
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>Ödeme seçeneklerim nelerdir?</t>
         </is>
       </c>
       <c r="I19" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/online-alisveris/odeme/odeme-seceneklerim-nelerdir</t>
         </is>
       </c>
       <c r="J19" s="19" t="n">
-        <v>5510</v>
+        <v>11454</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>7</v>
+        <v>944</v>
       </c>
       <c r="L19" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/islem-merkezi/hat-ozetim/hat-ozetim-nedir</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/servisler/arama-fatura-tl/turkcellmobilodeme</t>
         </is>
       </c>
     </row>
@@ -13240,12 +13270,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-kampanyalarimla-hangi-islemleri-yapabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarife-bilgilerimi-nasil-sorgularim</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
@@ -13263,28 +13293,28 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>Kampanyalarım Sayfasında Hangi İşlemleri Yapabilirim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="I20" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="J20" s="19" t="n">
-        <v>5152</v>
+        <v>6518</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="L20" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/islem-merkezi/hat-ozetim/hat-ozetim-nedir</t>
+          <t>301 ile yönlendirilmesi (sorgular genel paket ve tarife araması): https://www.turkcell.com.tr/paket-ve-tarifeler</t>
         </is>
       </c>
     </row>
@@ -13294,12 +13324,12 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/avans-tl-nedir-nasil-abone-olurum</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-servislerim-sayfasindan-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
@@ -13317,28 +13347,28 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>Avans TL Nedir? Nasıl Abone Olurum?</t>
+          <t>Servislerim Sayfasında Hangi Bilgiler Var?</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>Kendi numaramı nasıl gizleyebilirim?</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J21" s="19" t="n">
-        <v>4580</v>
+        <v>5510</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>98</v>
+        <v>7</v>
       </c>
       <c r="L21" s="14" t="inlineStr">
         <is>
-          <t>Servisin yayında olup olmadığının teyit edilmesi; yayında değilse 410 dönmesi</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell online işlemler'): https://www.turkcell.com.tr/destek/islem-merkezi</t>
         </is>
       </c>
     </row>
@@ -13348,12 +13378,12 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-nasil-tasiyabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/turkcell-hesabimda-kampanyalarimla-hangi-islemleri-yapabilirim</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
@@ -13371,28 +13401,28 @@
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>Numaramı Turkcell’e Taşımak için Ne Yapmalıyım?</t>
+          <t>Kampanyalarım Sayfasında Hangi İşlemleri Yapabilirim?</t>
         </is>
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>Numaramı taşımak ücretli midir?</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>4541</v>
+        <v>5152</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="L22" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-nasil-tasiyabilirim</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell online işlemler'): https://www.turkcell.com.tr/destek/islem-merkezi</t>
         </is>
       </c>
     </row>
@@ -13402,12 +13432,12 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tuketici-sikayetleri/sikayet-talebi-olusturma</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/avans-tl-nedir-nasil-abone-olurum</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
@@ -13425,28 +13455,28 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Avans TL Nedir? Nasıl Abone Olurum?</t>
         </is>
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
         </is>
       </c>
       <c r="J23" s="19" t="n">
-        <v>3123</v>
+        <v>4580</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>1614</v>
+        <v>98</v>
       </c>
       <c r="L23" s="14" t="inlineStr">
         <is>
-          <t>Şikayet formunun güncel adresinin teyit edilmesi ve bu adrese 301 ile yönlendirilmesi (sayfa bugün H1 ve title olmadan dönüyor)</t>
+          <t>410 dönmesi (Avans TL servis sayfası da kaldırılmış)</t>
         </is>
       </c>
     </row>
@@ -13456,12 +13486,12 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/nasil-hazirkart-alirim</t>
+          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-nasil-tasiyabilirim</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
@@ -13479,28 +13509,28 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>Nasıl faturalı hat alabilirim?</t>
+          <t>Numaramı Turkcell’e Taşımak için Ne Yapmalıyım?</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Nasıl faturalı hat alabilirim?</t>
+          <t>Numaramı taşımak ücretli midir?</t>
         </is>
       </c>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/nasil-faturali-hat-alabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
         </is>
       </c>
       <c r="J24" s="19" t="n">
-        <v>2934</v>
+        <v>4541</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="L24" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/nasil-hazirkart-alirim</t>
+          <t>301 ile yönlendirilmesi (sorgular Turkcell'e geçiş ve numara taşıma arıyor): https://www.turkcell.com.tr/turkcellli-olmak/paket-secimi</t>
         </is>
       </c>
     </row>
@@ -13510,12 +13540,12 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimlerine-nereden-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/nasil-hazirkart-alirim</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
@@ -13523,7 +13553,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
+          <t>Kendi adresi</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -13533,28 +13563,28 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>Nasıl faturalı hat alabilirim?</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>Nasıl faturalı hat alabilirim?</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/nasil-faturali-hat-alabilirim</t>
         </is>
       </c>
       <c r="J25" s="19" t="n">
-        <v>2481</v>
+        <v>2934</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi (bugün destek ana sayfasına yönleniyor)</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/nasil-hazirkart-alirim</t>
         </is>
       </c>
     </row>
@@ -13564,12 +13594,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kredi-transfer-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimlerine-nereden-ulasabilirim</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
@@ -13577,7 +13607,7 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -13587,28 +13617,28 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>Kredi Transfer Nedir? | Sıkça Sorulan Sorular</t>
+          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>Kendi numaramı nasıl gizleyebilirim?</t>
+          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
         </is>
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>1268</v>
+        <v>2481</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>242</v>
+        <v>108</v>
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/hazirkart/kreditransfer-nedir</t>
+          <t>301 ile Turkcell Akademi platformuna yönlendirilmesi (sorgular 'turkcell akademi'): https://tag.turkcell.com.tr/</t>
         </is>
       </c>
     </row>
@@ -13618,12 +13648,12 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kredi-transfer-nedir</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
@@ -13641,28 +13671,28 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
+          <t>Kredi Transfer Nedir? | Sıkça Sorulan Sorular</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
           <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>Kendi numaramı nasıl gizleyebilirim?</t>
-        </is>
-      </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
         </is>
       </c>
       <c r="J27" s="19" t="n">
-        <v>1227</v>
+        <v>1268</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>12</v>
+        <v>242</v>
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/servisler/arama-fatura-tl/turkcellmobilodeme</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/hazirkart/kreditransfer-nedir</t>
         </is>
       </c>
     </row>
@@ -13672,12 +13702,12 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
@@ -13695,28 +13725,28 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>Numaramı Taşırken Hattım Kullanıma Kapanır Mı?</t>
+          <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>Numaramı taşımak ücretli midir?</t>
+          <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
         </is>
       </c>
       <c r="J28" s="19" t="n">
-        <v>779</v>
+        <v>1227</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="L28" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
+          <t>301 ile yönlendirilmesi (sorgular 'telefonu kapalı gösterme', 'açıkken ulaşılamıyor'): https://www.turkcell.com.tr/servisler/arama-fatura-tl/yonlendir</t>
         </is>
       </c>
     </row>
@@ -13726,12 +13756,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
@@ -13749,28 +13779,28 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Paket ve Tarifelerim Sayfasında Neler Yapabilirim?</t>
+          <t>Numaramı Taşırken Hattım Kullanıma Kapanır Mı?</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>Numaramı taşımak ücretli midir?</t>
         </is>
       </c>
       <c r="I29" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>382</v>
+        <v>779</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
         </is>
       </c>
     </row>
@@ -13780,12 +13810,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/sosyal-destek-iletisim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
@@ -13803,28 +13833,28 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Paket ve Tarifelerim Sayfasında Neler Yapabilirim?</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J30" s="19" t="n">
-        <v>257</v>
+        <v>382</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="L30" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell online işlemler'): https://www.turkcell.com.tr/destek/islem-merkezi</t>
         </is>
       </c>
     </row>
@@ -13834,12 +13864,12 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/mevcut-egitimlerden-baska-egitimler-olacak-mi</t>
+          <t>https://www.turkcell.com.tr/destek/sosyal-destek-iletisim</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
@@ -13847,7 +13877,7 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
+          <t>Kendi adresi</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -13857,12 +13887,12 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
@@ -13871,14 +13901,14 @@
         </is>
       </c>
       <c r="J31" s="19" t="n">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi (bugün destek ana sayfasına yönleniyor)</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell sosyal destek'): https://www.turkcell.com.tr/sosyal-destek</t>
         </is>
       </c>
     </row>
@@ -13888,12 +13918,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/mevcut-egitimlerden-baska-egitimler-olacak-mi</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
@@ -13901,7 +13931,7 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -13911,28 +13941,28 @@
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>TL Ayarlarım Sayfasından Neler Yapabilirim?</t>
+          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
         </is>
       </c>
       <c r="I32" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J32" s="19" t="n">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="L32" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>301 ile Turkcell Akademi platformuna yönlendirilmesi (sorgular 'turkcell akademi'): https://tag.turkcell.com.tr/</t>
         </is>
       </c>
     </row>
@@ -13942,12 +13972,12 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 · yazım varyantı</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
@@ -13955,38 +13985,38 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>Kendi adresi</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>noindex,follow</t>
+          <t>index,follow</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>CLIP Özelliği Nedir? | Turkcell Destek</t>
+          <t>TL Ayarlarım Sayfasından Neler Yapabilirim?</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>Arayan numarayı göster (CLIP) özelliği nedir?</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J33" s="19" t="n">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>404 ya da 410 dönmesi (karşılayan sayfa yok)</t>
         </is>
       </c>
     </row>
@@ -13996,12 +14026,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="D34" s="11" t="n">
@@ -14009,38 +14039,38 @@
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>noindex,follow</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
+          <t>CLIP Özelliği Nedir? | Turkcell Destek</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
+          <t>Arayan numarayı göster (CLIP) özelliği nedir?</t>
         </is>
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="J34" s="19" t="n">
-        <v>55</v>
+        <v>129</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="L34" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
     </row>
@@ -14050,12 +14080,12 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
@@ -14073,28 +14103,28 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/hattim-fatura-borcu-nedeniyle-kapanirsa-yeniden-actirmak-icin-bir-ucret-oder-miyim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="J35" s="19" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L35" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
     </row>
@@ -14104,12 +14134,12 @@
       </c>
       <c r="B36" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris/turkcell-pasaj/turkcell-pasajda-satici-olmak-istiyorum-nereye-basvurabilirim</t>
+          <t>https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-</t>
         </is>
       </c>
       <c r="D36" s="11" t="n">
@@ -14122,33 +14152,33 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>noindex,nofollow</t>
+          <t>index,follow</t>
         </is>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Pasaj’da Satıcı Olmak İstiyorum, Nereye Başvurabilirim?</t>
+          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Pasaj'da satıcı olmak istiyorum.</t>
+          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/hattim-fatura-borcu-nedeniyle-kapanirsa-yeniden-actirmak-icin-bir-ucret-oder-miyim</t>
         </is>
       </c>
       <c r="J36" s="19" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L36" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>Kesik adresin sayfanın tam adresine 301 ile yönlendirilmesi: https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-gelen-ve-gelen-giden-iletisime-ne-kadar-sureyle-kapatabilirim-ve-faturama-herhangi-bir-ucret-yansir-m</t>
         </is>
       </c>
     </row>
@@ -14158,7 +14188,7 @@
       </c>
       <c r="B37" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -14202,7 +14232,7 @@
       </c>
       <c r="L37" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/abonelik-islemleri/hattimi-nasil-iptal-ettirebilirim</t>
         </is>
       </c>
     </row>
@@ -14212,7 +14242,7 @@
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 · yazım varyantı</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -14266,7 +14296,7 @@
       </c>
       <c r="B39" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 · yazım varyantı</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -14320,7 +14350,7 @@
       </c>
       <c r="B40" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -14374,7 +14404,7 @@
       </c>
       <c r="B41" s="22" t="inlineStr">
         <is>
-          <t>Soft 404</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -15870,7 +15900,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Aynı Başlığı Taşıyan Destek Sayfaları</t>
+          <t>Duplicate Adresler · Aynı Başlığı ve Cevabı Taşıyan Destek Sayfaları</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Soft 404 - tekrar eden sayfalar listesi 24 adrese indirildi (akademi, m. ve www'suz varyantlar cikarildi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
+++ b/Turkcell-Destek-Sayfa-Onerileri-22-09-2026.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Talepler'!$A$4:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Yeni Sayfa Önerileri'!$A$4:$U$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mevcut Sayfa Güçlendirme'!$A$4:$O$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sitemap Dışı Adresler'!$A$4:$L$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sitemap Dışı Adresler'!$A$4:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Doğrulanacak Bilgiler'!$A$4:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Duplicate Adresler'!$A$4:$G$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Rakip Karşılaştırması'!$A$4:$K$79</definedName>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Geçerli bir kategori ve alt bölüm altında yayında olmayan bir soru adresi istendiğinde sunucu 200 status code döndürmekte, alt bölümdeki başka bir sayfanın içeriğini göstermekte, adresin kendisine canonical vermekte ve index,follow taşımaktadır (test: /destek/tarife-ve-paketler/konusma/bu-sayfa-yok-deneme-xyz, 14 Eyl 2026). Geçersiz kategori ya da alt bölüm altında adres doğru biçimde 404 dönmektedir. Search Console'da 1 Eyl 2025 - 31 Ağu 2026 penceresinde bu davranışı gösteren 28 adres görülmüştür: 24 adres başka bir sayfanın içeriğini tekrar etmekte (212.184 impression, 5.168 tıklama), 4 adres ise gerçek bir sayfanın yazım varyantı olarak kopyasını sunmaktadır (95.306 impression). Toplam 307.490 impression. Şikayet talebi oluşturma ve Pasaj satıcı sayfaları kendi içeriğini gösterdiği için bu listeye alınmamıştır.</t>
+          <t>Geçerli bir kategori ve alt bölüm altında yayında olmayan bir soru adresi istendiğinde sunucu 200 status code döndürmekte, alt bölümdeki başka bir sayfanın içeriğini göstermekte, adresin kendisine canonical vermekte ve index,follow taşımaktadır (test: /destek/tarife-ve-paketler/konusma/bu-sayfa-yok-deneme-xyz, 14 Eyl 2026). Geçersiz kategori ya da alt bölüm altında adres doğru biçimde 404 dönmektedir. Search Console'da 1 Eyl 2025 - 31 Ağu 2026 penceresinde bu davranışı gösteren 24 adres görülmüştür: 21 adres başka bir sayfanın içeriğini tekrar etmekte (209.530 impression, 5.055 tıklama), 3 adres ise gerçek bir sayfanın yazım varyantı olarak kopyasını sunmaktadır (95.299 impression). Toplam 304.829 impression. Şikayet talebi oluşturma ve Pasaj satıcı sayfaları kendi içeriğini gösterdiği için bu listeye alınmamıştır.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>28 adres · 307.490 impression (Search Console, 1 Eyl 2025 - 31 Ağu 2026) + şablon kuralı</t>
+          <t>24 adres · 304.829 impression (Search Console, 1 Eyl 2025 - 31 Ağu 2026) + şablon kuralı</t>
         </is>
       </c>
     </row>
@@ -1785,22 +1785,18 @@
 /destek/servisler-ve-internet/servisler/avans-tl-nedir-nasil-abone-olurum · 4.580 impression → 410 dönmesi (Avans TL servis sayfası da kaldırılmış)
 /destek/kampanya/kampanyalar-faturali/numarami-nasil-tasiyabilirim · 4.541 impression → 301 → /turkcellli-olmak/paket-secimi
 /destek/turkcellli-olmak/turkcellli-olmak/nasil-hazirkart-alirim · 2.934 impression → 301 → /destek/turkcellli-olmak/numara-tasima/nasil-hazirkart-alirim
-/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimlerine-nereden-ulasabilirim · 2.481 impression → 301 → https://tag.turkcell.com.tr/
 /destek/servisler-ve-internet/servisler/kredi-transfer-nedir · 1.268 impression → 301 → /destek/hattiniz/hazirkart/kreditransfer-nedir
 /destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim · 1.227 impression → 301 → /servisler/arama-fatura-tl/yonlendir
 /destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi · 779 impression → 301 → /destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi
 /destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim · 382 impression → 301 → /destek/islem-merkezi
 /destek/sosyal-destek-iletisim · 257 impression → 301 → /sosyal-destek
-/destek/turkcell-akademi/sikca-sorulan-sorular/mevcut-egitimlerden-baska-egitimler-olacak-mi · 172 impression → 301 → https://tag.turkcell.com.tr/
 /destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim · 145 impression → 404 ya da 410 dönmesi (karşılayan sayfa yok)
 /destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir · 129 impression → 301 → /destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir
 /destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim · 55 impression → 301 → /destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim
 /kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak- · 33 impression → 301 → /kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-gelen-ve-gelen-giden-iletisime-ne-kadar-sureyle-kapatabilirim-ve-faturama-herhangi-bir-ucret-yansir-m
 /destek/islem-merkezi/ayarlarim/hat-iptalimi-nasil-gerceklestirebilirim · 14 impression → 301 → /destek/hattiniz/abonelik-islemleri/hattimi-nasil-iptal-ettirebilirim
 /destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken · 14 impression → 301 → /destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir
-/destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir · 7 impression → 301 → /destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir
-/destek/hizmet-kanallarimiz/musteri-hizmetleri/gencaver · 1 impression → 404 ya da 410 dönmesi
-/destek/online-alisveris · 1 impression → 301 → /destek/online-alisveris</t>
+/destek/hizmet-kanallarimiz/musteri-hizmetleri/gencaver · 1 impression → 404 ya da 410 dönmesi</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
@@ -12540,7 +12536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13857,7 +13853,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimlerine-nereden-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kredi-transfer-nedir</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
@@ -13865,7 +13861,7 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
+          <t>Kendi adresi</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -13875,28 +13871,28 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>Kredi Transfer Nedir? | Sıkça Sorulan Sorular</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>2481</v>
+        <v>1268</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>108</v>
+        <v>242</v>
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
-          <t>301 ile Turkcell Akademi platformuna yönlendirilmesi (sorgular 'turkcell akademi'): https://tag.turkcell.com.tr/</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/hazirkart/kreditransfer-nedir</t>
         </is>
       </c>
     </row>
@@ -13911,7 +13907,7 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kredi-transfer-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
@@ -13929,7 +13925,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>Kredi Transfer Nedir? | Sıkça Sorulan Sorular</t>
+          <t>Kendi numaramı nasıl gizleyebilirim?</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
@@ -13943,14 +13939,14 @@
         </is>
       </c>
       <c r="J27" s="19" t="n">
-        <v>1268</v>
+        <v>1227</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>242</v>
+        <v>12</v>
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/hazirkart/kreditransfer-nedir</t>
+          <t>301 ile yönlendirilmesi (sorgular 'telefonu kapalı gösterme', 'açıkken ulaşılamıyor'): https://www.turkcell.com.tr/servisler/arama-fatura-tl/yonlendir</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13961,7 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/telefonumu-mobil-odeme-kullanimina-nasil-acabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
@@ -13983,28 +13979,28 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>Kendi numaramı nasıl gizleyebilirim?</t>
+          <t>Numaramı Taşırken Hattım Kullanıma Kapanır Mı?</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>Kendi numaramı nasıl gizleyebilirim?</t>
+          <t>Numaramı taşımak ücretli midir?</t>
         </is>
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/servisler-ve-internet/servisler/kendi-numarami-nasil-gizleyebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
         </is>
       </c>
       <c r="J28" s="19" t="n">
-        <v>1227</v>
+        <v>779</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="L28" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi (sorgular 'telefonu kapalı gösterme', 'açıkken ulaşılamıyor'): https://www.turkcell.com.tr/servisler/arama-fatura-tl/yonlendir</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
         </is>
       </c>
     </row>
@@ -14019,7 +14015,7 @@
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/kampanya/kampanyalar-faturali/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
@@ -14037,28 +14033,28 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Numaramı Taşırken Hattım Kullanıma Kapanır Mı?</t>
+          <t>Paket ve Tarifelerim Sayfasında Neler Yapabilirim?</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>Numaramı taşımak ücretli midir?</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I29" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasimak-ucretli-midir</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>779</v>
+        <v>382</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/turkcellli-olmak/numara-tasima/numarami-tasirken-hattim-kullanima-kapanir-mi</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell online işlemler'): https://www.turkcell.com.tr/destek/islem-merkezi</t>
         </is>
       </c>
     </row>
@@ -14073,7 +14069,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/paket-ve-tarifelerim-sayfasindan-hangi-islemleri-yapabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/sosyal-destek-iletisim</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
@@ -14091,28 +14087,28 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>Paket ve Tarifelerim Sayfasında Neler Yapabilirim?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J30" s="19" t="n">
-        <v>382</v>
+        <v>257</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="L30" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi (sorgular 'turkcell online işlemler'): https://www.turkcell.com.tr/destek/islem-merkezi</t>
+          <t>301 ile yönlendirilmesi (sorgular 'turkcell sosyal destek'): https://www.turkcell.com.tr/sosyal-destek</t>
         </is>
       </c>
     </row>
@@ -14127,7 +14123,7 @@
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/sosyal-destek-iletisim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
@@ -14145,28 +14141,28 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TL Ayarlarım Sayfasından Neler Yapabilirim?</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
         </is>
       </c>
       <c r="J31" s="19" t="n">
-        <v>257</v>
+        <v>145</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi (sorgular 'turkcell sosyal destek'): https://www.turkcell.com.tr/sosyal-destek</t>
+          <t>404 ya da 410 dönmesi (karşılayan sayfa yok)</t>
         </is>
       </c>
     </row>
@@ -14176,12 +14172,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 - tekrar eden sayfa</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/mevcut-egitimlerden-baska-egitimler-olacak-mi</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
@@ -14189,38 +14185,38 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Yönleniyor: https://www.turkcell.com.tr/destek</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>noindex,follow</t>
         </is>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Destek - Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>CLIP Özelliği Nedir? | Turkcell Destek</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>Merhaba, Size Nasıl Yardımcı Olabiliriz?</t>
+          <t>Arayan numarayı göster (CLIP) özelliği nedir?</t>
         </is>
       </c>
       <c r="I32" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
       <c r="J32" s="19" t="n">
-        <v>172</v>
+        <v>129</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="L32" s="14" t="inlineStr">
         <is>
-          <t>301 ile Turkcell Akademi platformuna yönlendirilmesi (sorgular 'turkcell akademi'): https://tag.turkcell.com.tr/</t>
+          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
         </is>
       </c>
     </row>
@@ -14235,7 +14231,7 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/tl-ayarlarim-sayfasindan-hangi-ayarlari-yapabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
@@ -14253,28 +14249,28 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>TL Ayarlarım Sayfasından Neler Yapabilirim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>Hat Özetimde hattım ile ilgili hangi bilgilere ulaşabilirim?</t>
+          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/islem-merkezinden-yapilabilen-online-islemler/hat-ozetimde-hattim-ile-ilgili-hangi-bilgilere-ulasabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
       <c r="J33" s="19" t="n">
-        <v>145</v>
+        <v>55</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi (karşılayan sayfa yok)</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
         </is>
       </c>
     </row>
@@ -14284,12 +14280,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
+          <t>Soft 404 - tekrar eden sayfa</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-</t>
         </is>
       </c>
       <c r="D34" s="11" t="n">
@@ -14297,38 +14293,38 @@
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>Kendi adresi</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>noindex,follow</t>
+          <t>index,follow</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>CLIP Özelliği Nedir? | Turkcell Destek</t>
+          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>Arayan numarayı göster (CLIP) özelliği nedir?</t>
+          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
         </is>
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcellli-olmak/turkcellli-olmak/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/hattim-fatura-borcu-nedeniyle-kapanirsa-yeniden-actirmak-icin-bir-ucret-oder-miyim</t>
         </is>
       </c>
       <c r="J34" s="19" t="n">
-        <v>129</v>
+        <v>33</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="L34" s="14" t="inlineStr">
         <is>
-          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/sikca-sorulan-sorular/arayan-numarayi-goster-clip-ozelligi-nedir</t>
+          <t>Kesik adresin sayfanın tam adresine 301 ile yönlendirilmesi: https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-gelen-ve-gelen-giden-iletisime-ne-kadar-sureyle-kapatabilirim-ve-faturama-herhangi-bir-ucret-yansir-m</t>
         </is>
       </c>
     </row>
@@ -14343,7 +14339,7 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nerden-ogrenebilirim-ve-nasil-degistirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/hat-iptalimi-nasil-gerceklestirebilirim</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
@@ -14361,28 +14357,28 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
+          <t>Profil bilgilerim nedir?</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Paket / Tarife değişikliğini nasıl yapabilirim?</t>
+          <t>Profil bilgilerim nedir?</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/profil-bilgilerim-nedir</t>
         </is>
       </c>
       <c r="J35" s="19" t="n">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L35" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/tarife-ve-paketler/konusma/tarifemi-nasil-degistirebilirim</t>
+          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/abonelik-islemleri/hattimi-nasil-iptal-ettirebilirim</t>
         </is>
       </c>
     </row>
@@ -14392,12 +14388,12 @@
       </c>
       <c r="B36" s="22" t="inlineStr">
         <is>
-          <t>Soft 404 - tekrar eden sayfa</t>
+          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-</t>
+          <t>https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken</t>
         </is>
       </c>
       <c r="D36" s="11" t="n">
@@ -14415,28 +14411,28 @@
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
+          <t>Financell kredi taksitlerim dışında ödemem gereken diğer ücretler nelerdir?</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Hattım fatura borcu nedeniyle kapanırsa, yeniden kapama/açma için bir ücret öder miyim?</t>
+          <t>Financell kredi taksitlerim dışında ödemem gereken diğer ücretler nelerdir?</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hattiniz/faturali/hattim-fatura-borcu-nedeniyle-kapanirsa-yeniden-actirmak-icin-bir-ucret-oder-miyim</t>
+          <t>https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir</t>
         </is>
       </c>
       <c r="J36" s="19" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L36" s="14" t="inlineStr">
         <is>
-          <t>Kesik adresin sayfanın tam adresine 301 ile yönlendirilmesi: https://www.turkcell.com.tr/kurumsal/destek/hattiniz/faturali/hattimi-gecici-olarak-gelen-ve-gelen-giden-iletisime-ne-kadar-sureyle-kapatabilirim-ve-faturama-herhangi-bir-ucret-yansir-m</t>
+          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir</t>
         </is>
       </c>
     </row>
@@ -14451,7 +14447,7 @@
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/hat-iptalimi-nasil-gerceklestirebilirim</t>
+          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/gencaver</t>
         </is>
       </c>
       <c r="D37" s="11" t="n">
@@ -14469,28 +14465,28 @@
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>Profil bilgilerim nedir?</t>
+          <t>Turkcell Hizmet</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>Profil bilgilerim nedir?</t>
+          <t>Turkcell Hizmet</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/islem-merkezi/ayarlarim/profil-bilgilerim-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/turkcell-hizmet</t>
         </is>
       </c>
       <c r="J37" s="19" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" s="14" t="inlineStr">
         <is>
-          <t>301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/hattiniz/abonelik-islemleri/hattimi-nasil-iptal-ettirebilirim</t>
+          <t>404 ya da 410 dönmesi</t>
         </is>
       </c>
     </row>
@@ -14498,53 +14494,53 @@
       <c r="A38" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>404 · kaldırılmış</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-nedir</t>
         </is>
       </c>
       <c r="D38" s="11" t="n">
-        <v>200</v>
+        <v>404</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>Financell kredi taksitlerim dışında ödemem gereken diğer ücretler nelerdir?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>Financell kredi taksitlerim dışında ödemem gereken diğer ücretler nelerdir?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I38" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J38" s="19" t="n">
-        <v>14</v>
+        <v>17389</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="L38" s="14" t="inlineStr">
         <is>
-          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/financell/ucretlendirme/financell-kredi-taksitlerim-disinda-odemem-gereken-diger-ucretler-nelerdir</t>
+          <t>İşlem gerekmiyor</t>
         </is>
       </c>
     </row>
@@ -14552,53 +14548,53 @@
       <c r="A39" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404 - tekrar eden sayfa · yazım varyantı</t>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>404 · kaldırılmış</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/bazi-egitimleri-izlemeye-calistigimda-hizli-giris-ile-giris-yapmam-isteniyor-neden</t>
         </is>
       </c>
       <c r="D39" s="11" t="n">
-        <v>200</v>
+        <v>404</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>Online Alışverişlerde Paycell Alışveriş Limiti Nasıl Kullanılır?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>Online alışverişlerde Paycell Alışveriş Limiti nasıl kullanılır?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I39" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J39" s="19" t="n">
-        <v>7</v>
+        <v>2744</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>0</v>
+        <v>481</v>
       </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>Doğru adrese 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/financell/paycell-alisveris-limiti/online-alisverislerde-paycell-alisveris-limiti-nasil-kullanilir</t>
+          <t>İşlem gerekmiyor</t>
         </is>
       </c>
     </row>
@@ -14606,53 +14602,53 @@
       <c r="A40" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404 - tekrar eden sayfa</t>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>404 · kaldırılmış</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/gencaver</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/coursera-nedir</t>
         </is>
       </c>
       <c r="D40" s="11" t="n">
-        <v>200</v>
+        <v>404</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Hizmet</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Hizmet</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I40" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/hizmet-kanallarimiz/musteri-hizmetleri/turkcell-hizmet</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J40" s="19" t="n">
-        <v>1</v>
+        <v>1703</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L40" s="14" t="inlineStr">
         <is>
-          <t>404 ya da 410 dönmesi</t>
+          <t>İşlem gerekmiyor</t>
         </is>
       </c>
     </row>
@@ -14660,53 +14656,53 @@
       <c r="A41" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="22" t="inlineStr">
-        <is>
-          <t>Soft 404 - tekrar eden sayfa</t>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>404 · kaldırılmış</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademide-hangi-tur-egitimler-bulabilirim</t>
         </is>
       </c>
       <c r="D41" s="11" t="n">
-        <v>200</v>
+        <v>404</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>Kendi adresi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>index,follow</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Pasaj'da Online Alışveriş | Turkcell Destek</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>Turkcell Pasaj</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/online-alisveris</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J41" s="19" t="n">
-        <v>1</v>
+        <v>740</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>1</v>
+        <v>103</v>
       </c>
       <c r="L41" s="14" t="inlineStr">
         <is>
-          <t>m. alt alan adının www adresine 301 ile yönlendirilmesi: https://www.turkcell.com.tr/destek/online-alisveris</t>
+          <t>İşlem gerekmiyor</t>
         </is>
       </c>
     </row>
@@ -14721,7 +14717,7 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/istedigim-egitime-nasil-kayit-yaparim</t>
         </is>
       </c>
       <c r="D42" s="11" t="n">
@@ -14753,10 +14749,10 @@
         </is>
       </c>
       <c r="J42" s="19" t="n">
-        <v>17389</v>
+        <v>580</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>420</v>
+        <v>78</v>
       </c>
       <c r="L42" s="14" t="inlineStr">
         <is>
@@ -14775,7 +14771,7 @@
       </c>
       <c r="C43" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/bazi-egitimleri-izlemeye-calistigimda-hizli-giris-ile-giris-yapmam-isteniyor-neden</t>
+          <t>https://www.turkcell.com.tr/destek/wiyo/dask/zorunlu-deprem-sigortasi-gecerlilik-suresi-ne-kadardir</t>
         </is>
       </c>
       <c r="D43" s="11" t="n">
@@ -14807,10 +14803,10 @@
         </is>
       </c>
       <c r="J43" s="19" t="n">
-        <v>2744</v>
+        <v>287</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>481</v>
+        <v>3</v>
       </c>
       <c r="L43" s="14" t="inlineStr">
         <is>
@@ -14829,7 +14825,7 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/coursera-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/program-nedir</t>
         </is>
       </c>
       <c r="D44" s="11" t="n">
@@ -14861,10 +14857,10 @@
         </is>
       </c>
       <c r="J44" s="19" t="n">
-        <v>1703</v>
+        <v>150</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="L44" s="14" t="inlineStr">
         <is>
@@ -14883,7 +14879,7 @@
       </c>
       <c r="C45" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademide-hangi-tur-egitimler-bulabilirim</t>
+          <t>https://www.turkcell.com.tr/destek/wiyo/dask/dask-zorunlu-deprem-sigortasi-nedir</t>
         </is>
       </c>
       <c r="D45" s="11" t="n">
@@ -14915,10 +14911,10 @@
         </is>
       </c>
       <c r="J45" s="19" t="n">
-        <v>740</v>
+        <v>132</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="L45" s="14" t="inlineStr">
         <is>
@@ -14937,7 +14933,7 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/istedigim-egitime-nasil-kayit-yaparim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-ile-courseranin-nasil-bir-isbirligi-var</t>
         </is>
       </c>
       <c r="D46" s="11" t="n">
@@ -14969,10 +14965,10 @@
         </is>
       </c>
       <c r="J46" s="19" t="n">
-        <v>580</v>
+        <v>108</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="L46" s="14" t="inlineStr">
         <is>
@@ -14991,7 +14987,7 @@
       </c>
       <c r="C47" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/wiyo/dask/zorunlu-deprem-sigortasi-gecerlilik-suresi-ne-kadardir</t>
+          <t>https://www.turkcell.com.tr/destek/wiyo/dask/dask-zorunlu-deprem-sigortasi-primini-belirleyen-faktorler-nelerdir</t>
         </is>
       </c>
       <c r="D47" s="11" t="n">
@@ -15023,10 +15019,10 @@
         </is>
       </c>
       <c r="J47" s="19" t="n">
-        <v>287</v>
+        <v>90</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L47" s="14" t="inlineStr">
         <is>
@@ -15045,7 +15041,7 @@
       </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/program-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/coursera-egitimleri-ucretli-mi</t>
         </is>
       </c>
       <c r="D48" s="11" t="n">
@@ -15077,10 +15073,10 @@
         </is>
       </c>
       <c r="J48" s="19" t="n">
-        <v>150</v>
+        <v>26</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L48" s="14" t="inlineStr">
         <is>
@@ -15099,7 +15095,7 @@
       </c>
       <c r="C49" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/wiyo/dask/dask-zorunlu-deprem-sigortasi-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/egitime-kayit-oldum-ancak-icerikler-ingilizce-nasil-ilerlemeliyim</t>
         </is>
       </c>
       <c r="D49" s="11" t="n">
@@ -15131,10 +15127,10 @@
         </is>
       </c>
       <c r="J49" s="19" t="n">
-        <v>132</v>
+        <v>19</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="14" t="inlineStr">
         <is>
@@ -15153,7 +15149,7 @@
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-ile-courseranin-nasil-bir-isbirligi-var</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/izleyeceklerime-ekle-nedir</t>
         </is>
       </c>
       <c r="D50" s="11" t="n">
@@ -15185,10 +15181,10 @@
         </is>
       </c>
       <c r="J50" s="19" t="n">
-        <v>108</v>
+        <v>15</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L50" s="14" t="inlineStr">
         <is>
@@ -15207,7 +15203,7 @@
       </c>
       <c r="C51" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/wiyo/dask/dask-zorunlu-deprem-sigortasi-primini-belirleyen-faktorler-nelerdir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/devam-eden-egitimler-nedir</t>
         </is>
       </c>
       <c r="D51" s="11" t="n">
@@ -15239,10 +15235,10 @@
         </is>
       </c>
       <c r="J51" s="19" t="n">
-        <v>90</v>
+        <v>13</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L51" s="14" t="inlineStr">
         <is>
@@ -15261,7 +15257,7 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/coursera-egitimleri-ucretli-mi</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/egitimleri-izlemek-icin-gereksinimler-nelerdir</t>
         </is>
       </c>
       <c r="D52" s="11" t="n">
@@ -15293,10 +15289,10 @@
         </is>
       </c>
       <c r="J52" s="19" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L52" s="14" t="inlineStr">
         <is>
@@ -15315,7 +15311,7 @@
       </c>
       <c r="C53" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/egitime-kayit-oldum-ancak-icerikler-ingilizce-nasil-ilerlemeliyim</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/isaret-dili-ile-anlatim-iceren-egitimlere-nasil-ulasabilirim</t>
         </is>
       </c>
       <c r="D53" s="11" t="n">
@@ -15347,7 +15343,7 @@
         </is>
       </c>
       <c r="J53" s="19" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="K53" s="19" t="n">
         <v>1</v>
@@ -15369,7 +15365,7 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/izleyeceklerime-ekle-nedir</t>
+          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimleri-veya-portaliyle-ilgili-goruslerimi-nasil-iletebilirim</t>
         </is>
       </c>
       <c r="D54" s="11" t="n">
@@ -15401,7 +15397,7 @@
         </is>
       </c>
       <c r="J54" s="19" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K54" s="19" t="n">
         <v>1</v>
@@ -15412,224 +15408,8 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11" t="n">
-        <v>51</v>
-      </c>
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>404 · kaldırılmış</t>
-        </is>
-      </c>
-      <c r="C55" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/devam-eden-egitimler-nedir</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n">
-        <v>404</v>
-      </c>
-      <c r="E55" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I55" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J55" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="K55" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="L55" s="14" t="inlineStr">
-        <is>
-          <t>İşlem gerekmiyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="11" t="n">
-        <v>52</v>
-      </c>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>404 · kaldırılmış</t>
-        </is>
-      </c>
-      <c r="C56" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/egitimleri-izlemek-icin-gereksinimler-nelerdir</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n">
-        <v>404</v>
-      </c>
-      <c r="E56" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I56" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J56" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="K56" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="14" t="inlineStr">
-        <is>
-          <t>İşlem gerekmiyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="11" t="n">
-        <v>53</v>
-      </c>
-      <c r="B57" s="23" t="inlineStr">
-        <is>
-          <t>404 · kaldırılmış</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/isaret-dili-ile-anlatim-iceren-egitimlere-nasil-ulasabilirim</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n">
-        <v>404</v>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F57" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H57" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I57" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J57" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K57" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L57" s="14" t="inlineStr">
-        <is>
-          <t>İşlem gerekmiyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="n">
-        <v>54</v>
-      </c>
-      <c r="B58" s="23" t="inlineStr">
-        <is>
-          <t>404 · kaldırılmış</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/destek/turkcell-akademi/sikca-sorulan-sorular/turkcell-akademi-egitimleri-veya-portaliyle-ilgili-goruslerimi-nasil-iletebilirim</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="n">
-        <v>404</v>
-      </c>
-      <c r="E58" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I58" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J58" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K58" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L58" s="14" t="inlineStr">
-        <is>
-          <t>İşlem gerekmiyor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L58"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>

</xml_diff>